<commit_message>
set up per estrazione procedure
</commit_message>
<xml_diff>
--- a/i_test/test_D3_coorte_con_caratterizzazione/antidiabother.xlsx
+++ b/i_test/test_D3_coorte_con_caratterizzazione/antidiabother.xlsx
@@ -22,10 +22,10 @@
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
 <sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4" uniqueCount="4">
   <si>
-    <t xml:space="preserve">id</t>
-  </si>
-  <si>
-    <t xml:space="preserve">datasped</t>
+    <t xml:space="preserve">ID</t>
+  </si>
+  <si>
+    <t xml:space="preserve">DATE</t>
   </si>
   <si>
     <t xml:space="preserve">P01</t>

</xml_diff>